<commit_message>
Cerrar NA0 matematica y el universo precursor
</commit_message>
<xml_diff>
--- a/dominios/inmunologia/cambio-rumbo/03-base-documental-candidata/05-normalizacion-atomica-en-evaluacion/Registro_precursor_parametros_INMUNO_v0.1_2026-09-02.xlsx
+++ b/dominios/inmunologia/cambio-rumbo/03-base-documental-candidata/05-normalizacion-atomica-en-evaluacion/Registro_precursor_parametros_INMUNO_v0.1_2026-09-02.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="Re033f5cbeaf9446d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidatos_G2" sheetId="2" r:id="Rfe1146eb508e4859"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilotos_50" sheetId="3" r:id="R9e02e4fdd26a40e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colisiones_8" sheetId="4" r:id="Rc29b88f33e66473c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas" sheetId="5" r:id="Ra052f80d182541c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R69139af222b74880"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidatos_G2" sheetId="2" r:id="R87242cf52d934db7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pilotos_50" sheetId="3" r:id="R7b1162d99b4849f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colisiones_8" sheetId="4" r:id="Ra751acae3a4b401c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reglas" sheetId="5" r:id="Refeb15f8c986409f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -869,7 +869,7 @@
         <x:v>Cierre semántico</x:v>
       </x:c>
       <x:c r="I1" s="35" t="str">
-        <x:v>Estatuto atómico</x:v>
+        <x:v>Estado previo a adjudicación</x:v>
       </x:c>
       <x:c r="J1" s="35" t="str">
         <x:v>Observables</x:v>
@@ -1922,7 +1922,7 @@
         <x:v>G2-S2</x:v>
       </x:c>
       <x:c r="H25" s="28" t="str">
-        <x:v>PENDIENTE_AUDITORIA_EXTERNA</x:v>
+        <x:v>CERRADO_SEMANTICAMENTE</x:v>
       </x:c>
       <x:c r="I25" s="38" t="str">
         <x:v>CANDIDATO_NO_ADJUDICADO</x:v>
@@ -1966,7 +1966,7 @@
         <x:v>G2-S2</x:v>
       </x:c>
       <x:c r="H26" s="28" t="str">
-        <x:v>PENDIENTE_AUDITORIA_EXTERNA</x:v>
+        <x:v>CERRADO_SEMANTICAMENTE</x:v>
       </x:c>
       <x:c r="I26" s="38" t="str">
         <x:v>CANDIDATO_NO_ADJUDICADO</x:v>
@@ -2010,7 +2010,7 @@
         <x:v>G2-S2</x:v>
       </x:c>
       <x:c r="H27" s="28" t="str">
-        <x:v>PENDIENTE_AUDITORIA_EXTERNA</x:v>
+        <x:v>CERRADO_SEMANTICAMENTE</x:v>
       </x:c>
       <x:c r="I27" s="38" t="str">
         <x:v>CANDIDATO_NO_ADJUDICADO</x:v>
@@ -2054,7 +2054,7 @@
         <x:v>G2-S2</x:v>
       </x:c>
       <x:c r="H28" s="28" t="str">
-        <x:v>PENDIENTE_AUDITORIA_EXTERNA</x:v>
+        <x:v>CERRADO_SEMANTICAMENTE</x:v>
       </x:c>
       <x:c r="I28" s="38" t="str">
         <x:v>CANDIDATO_NO_ADJUDICADO</x:v>
@@ -2098,7 +2098,7 @@
         <x:v>G2-S2</x:v>
       </x:c>
       <x:c r="H29" s="28" t="str">
-        <x:v>PENDIENTE_AUDITORIA_EXTERNA</x:v>
+        <x:v>CERRADO_SEMANTICAMENTE</x:v>
       </x:c>
       <x:c r="I29" s="38" t="str">
         <x:v>CANDIDATO_NO_ADJUDICADO</x:v>
@@ -2142,7 +2142,7 @@
         <x:v>G2-S2</x:v>
       </x:c>
       <x:c r="H30" s="28" t="str">
-        <x:v>PENDIENTE_AUDITORIA_EXTERNA</x:v>
+        <x:v>CERRADO_SEMANTICAMENTE</x:v>
       </x:c>
       <x:c r="I30" s="38" t="str">
         <x:v>CANDIDATO_NO_ADJUDICADO</x:v>
@@ -2186,7 +2186,7 @@
         <x:v>G2-S2</x:v>
       </x:c>
       <x:c r="H31" s="28" t="str">
-        <x:v>PENDIENTE_AUDITORIA_EXTERNA</x:v>
+        <x:v>CERRADO_SEMANTICAMENTE</x:v>
       </x:c>
       <x:c r="I31" s="38" t="str">
         <x:v>CANDIDATO_NO_ADJUDICADO</x:v>
@@ -2230,7 +2230,7 @@
         <x:v>G2-S2</x:v>
       </x:c>
       <x:c r="H32" s="28" t="str">
-        <x:v>PENDIENTE_AUDITORIA_EXTERNA</x:v>
+        <x:v>CERRADO_SEMANTICAMENTE</x:v>
       </x:c>
       <x:c r="I32" s="38" t="str">
         <x:v>CANDIDATO_NO_ADJUDICADO</x:v>
@@ -2274,7 +2274,7 @@
         <x:v>G2-S2</x:v>
       </x:c>
       <x:c r="H33" s="28" t="str">
-        <x:v>PENDIENTE_AUDITORIA_EXTERNA</x:v>
+        <x:v>CERRADO_SEMANTICAMENTE</x:v>
       </x:c>
       <x:c r="I33" s="38" t="str">
         <x:v>CANDIDATO_NO_ADJUDICADO</x:v>
@@ -2298,7 +2298,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67b497115a344f3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a9f6155a4f3440c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3646,7 +3646,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb600465c4cfa4881"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b55a21d8ef44e21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3846,7 +3846,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68a7be132c3a4f8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f7472f6dd1e4c47"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>